<commit_message>
Hoan tat don dep: Luu font va khung thanh cuộn
</commit_message>
<xml_diff>
--- a/phan_giao.xlsx
+++ b/phan_giao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pxvanhanh/TPM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D0963F-4A09-594F-B0C5-19E62AFF86D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6FAE902-A9F2-BE4D-AF32-F11952D8E30C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -453,9 +453,6 @@
     <t>BM.P4.15.49</t>
   </si>
   <si>
-    <t>Dương Đăng Tiến</t>
-  </si>
-  <si>
     <t>HỆ THÔNG ĐIỀU HÒA TẠI CNN</t>
   </si>
   <si>
@@ -543,6 +540,9 @@
   </si>
   <si>
     <t>Nguyễn Dăng Kiên</t>
+  </si>
+  <si>
+    <t>Dương Dăng Tiến</t>
   </si>
 </sst>
 </file>
@@ -789,10 +789,19 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -805,17 +814,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1069,11 +1069,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="16">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="23"/>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="22" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="23"/>
@@ -1105,7 +1105,7 @@
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="24" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="23"/>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="5" spans="1:26" ht="17">
       <c r="A5" s="1"/>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="25" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="23"/>
@@ -1149,7 +1149,7 @@
       <c r="L5" s="4"/>
     </row>
     <row r="6" spans="1:26" ht="55.5" customHeight="1">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="26" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="23"/>
@@ -1360,7 +1360,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>32</v>
@@ -1388,7 +1388,7 @@
         <v>25</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>32</v>
@@ -1416,7 +1416,7 @@
         <v>25</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>38</v>
@@ -1444,7 +1444,7 @@
         <v>25</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>38</v>
@@ -1528,7 +1528,7 @@
         <v>25</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>48</v>
@@ -1643,7 +1643,7 @@
         <v>52</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G23" s="21">
         <v>1</v>
@@ -1671,7 +1671,7 @@
         <v>52</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G24" s="21">
         <v>1</v>
@@ -1696,7 +1696,7 @@
         <v>51</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F25" s="16" t="s">
         <v>16</v>
@@ -1724,7 +1724,7 @@
         <v>51</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F26" s="16" t="s">
         <v>16</v>
@@ -1780,7 +1780,7 @@
         <v>51</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F28" s="17" t="s">
         <v>26</v>
@@ -1808,7 +1808,7 @@
         <v>51</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F29" s="17" t="s">
         <v>26</v>
@@ -1836,10 +1836,10 @@
         <v>74</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G30" s="21">
         <v>5</v>
@@ -1867,7 +1867,7 @@
         <v>77</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G31" s="21">
         <v>1</v>
@@ -1892,7 +1892,7 @@
         <v>51</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F32" s="16" t="s">
         <v>16</v>
@@ -1920,7 +1920,7 @@
         <v>51</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F33" s="17" t="s">
         <v>37</v>
@@ -1951,7 +1951,7 @@
         <v>84</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G34" s="21">
         <v>2</v>
@@ -1979,7 +1979,7 @@
         <v>84</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G35" s="21">
         <v>2</v>
@@ -2007,7 +2007,7 @@
         <v>89</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G36" s="21">
         <v>5</v>
@@ -2035,7 +2035,7 @@
         <v>89</v>
       </c>
       <c r="F37" s="17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G37" s="21">
         <v>5</v>
@@ -2088,7 +2088,7 @@
         <v>74</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F39" s="20" t="s">
         <v>55</v>
@@ -2116,7 +2116,7 @@
         <v>74</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F40" s="20" t="s">
         <v>52</v>
@@ -2175,7 +2175,7 @@
         <v>100</v>
       </c>
       <c r="F42" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G42" s="21">
         <v>3</v>
@@ -2203,7 +2203,7 @@
         <v>105</v>
       </c>
       <c r="F43" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G43" s="21">
         <v>3</v>
@@ -2315,7 +2315,7 @@
         <v>100</v>
       </c>
       <c r="F47" s="17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G47" s="21">
         <v>3</v>
@@ -2371,7 +2371,7 @@
         <v>117</v>
       </c>
       <c r="F49" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G49" s="21">
         <v>6</v>
@@ -2399,7 +2399,7 @@
         <v>122</v>
       </c>
       <c r="F50" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G50" s="21">
         <v>1</v>
@@ -2455,7 +2455,7 @@
         <v>105</v>
       </c>
       <c r="F52" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G52" s="21">
         <v>3</v>
@@ -2483,7 +2483,7 @@
         <v>129</v>
       </c>
       <c r="F53" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G53" s="21">
         <v>3</v>
@@ -2539,7 +2539,7 @@
         <v>129</v>
       </c>
       <c r="F55" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G55" s="21">
         <v>5</v>
@@ -2564,7 +2564,7 @@
         <v>74</v>
       </c>
       <c r="E56" s="20" t="s">
-        <v>136</v>
+        <v>163</v>
       </c>
       <c r="F56" s="17" t="s">
         <v>52</v>
@@ -2583,10 +2583,10 @@
         <v>50</v>
       </c>
       <c r="B57" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C57" s="19" t="s">
         <v>137</v>
-      </c>
-      <c r="C57" s="19" t="s">
-        <v>138</v>
       </c>
       <c r="D57" s="19" t="s">
         <v>74</v>
@@ -2595,7 +2595,7 @@
         <v>129</v>
       </c>
       <c r="F57" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G57" s="21">
         <v>1</v>
@@ -2611,19 +2611,19 @@
         <v>51</v>
       </c>
       <c r="B58" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="C58" s="19" t="s">
         <v>139</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>140</v>
       </c>
       <c r="D58" s="19" t="s">
         <v>74</v>
       </c>
       <c r="E58" s="20" t="s">
-        <v>136</v>
+        <v>163</v>
       </c>
       <c r="F58" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G58" s="21">
         <v>4</v>
@@ -2639,10 +2639,10 @@
         <v>52</v>
       </c>
       <c r="B59" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="C59" s="19" t="s">
         <v>141</v>
-      </c>
-      <c r="C59" s="19" t="s">
-        <v>142</v>
       </c>
       <c r="D59" s="19" t="s">
         <v>74</v>
@@ -2667,16 +2667,16 @@
         <v>53</v>
       </c>
       <c r="B60" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="C60" s="19" t="s">
         <v>143</v>
-      </c>
-      <c r="C60" s="19" t="s">
-        <v>144</v>
       </c>
       <c r="D60" s="19" t="s">
         <v>74</v>
       </c>
       <c r="E60" s="20" t="s">
-        <v>136</v>
+        <v>163</v>
       </c>
       <c r="F60" s="17" t="s">
         <v>43</v>
@@ -2695,10 +2695,10 @@
         <v>54</v>
       </c>
       <c r="B61" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C61" s="19" t="s">
         <v>145</v>
-      </c>
-      <c r="C61" s="19" t="s">
-        <v>146</v>
       </c>
       <c r="D61" s="19" t="s">
         <v>74</v>
@@ -2707,7 +2707,7 @@
         <v>84</v>
       </c>
       <c r="F61" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G61" s="21">
         <v>4</v>
@@ -2723,10 +2723,10 @@
         <v>55</v>
       </c>
       <c r="B62" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C62" s="19" t="s">
         <v>147</v>
-      </c>
-      <c r="C62" s="19" t="s">
-        <v>148</v>
       </c>
       <c r="D62" s="19" t="s">
         <v>74</v>
@@ -2735,7 +2735,7 @@
         <v>84</v>
       </c>
       <c r="F62" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G62" s="21">
         <v>1</v>
@@ -2751,16 +2751,16 @@
         <v>56</v>
       </c>
       <c r="B63" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="C63" s="19" t="s">
         <v>149</v>
-      </c>
-      <c r="C63" s="19" t="s">
-        <v>150</v>
       </c>
       <c r="D63" s="19" t="s">
         <v>74</v>
       </c>
       <c r="E63" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F63" s="17" t="s">
         <v>26</v>
@@ -2779,19 +2779,19 @@
         <v>57</v>
       </c>
       <c r="B64" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C64" s="19" t="s">
         <v>151</v>
-      </c>
-      <c r="C64" s="19" t="s">
-        <v>152</v>
       </c>
       <c r="D64" s="19" t="s">
         <v>74</v>
       </c>
       <c r="E64" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F64" s="20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G64" s="21">
         <v>6</v>
@@ -2817,8 +2817,8 @@
       <c r="L65" s="3"/>
     </row>
     <row r="66" spans="1:12" ht="186.75" customHeight="1">
-      <c r="A66" s="24" t="s">
-        <v>153</v>
+      <c r="A66" s="27" t="s">
+        <v>152</v>
       </c>
       <c r="B66" s="23"/>
       <c r="C66" s="23"/>
@@ -2833,13 +2833,13 @@
       <c r="L66" s="3"/>
     </row>
     <row r="67" spans="1:12" ht="16">
-      <c r="A67" s="27" t="s">
-        <v>154</v>
+      <c r="A67" s="30" t="s">
+        <v>153</v>
       </c>
       <c r="B67" s="23"/>
       <c r="C67" s="23"/>
-      <c r="D67" s="25" t="s">
-        <v>155</v>
+      <c r="D67" s="28" t="s">
+        <v>154</v>
       </c>
       <c r="E67" s="23"/>
       <c r="F67" s="23"/>
@@ -2851,11 +2851,11 @@
       <c r="L67" s="4"/>
     </row>
     <row r="68" spans="1:12" ht="16">
-      <c r="A68" s="22"/>
+      <c r="A68" s="31"/>
       <c r="B68" s="23"/>
       <c r="C68" s="23"/>
-      <c r="D68" s="26" t="s">
-        <v>156</v>
+      <c r="D68" s="29" t="s">
+        <v>155</v>
       </c>
       <c r="E68" s="23"/>
       <c r="F68" s="23"/>
@@ -2868,7 +2868,7 @@
     </row>
     <row r="69" spans="1:12" ht="16">
       <c r="A69" s="2"/>
-      <c r="B69" s="22"/>
+      <c r="B69" s="31"/>
       <c r="C69" s="23"/>
       <c r="D69" s="2"/>
       <c r="E69" s="3"/>
@@ -2882,7 +2882,7 @@
     </row>
     <row r="70" spans="1:12" ht="16">
       <c r="A70" s="2"/>
-      <c r="B70" s="22"/>
+      <c r="B70" s="31"/>
       <c r="C70" s="23"/>
       <c r="D70" s="2"/>
       <c r="E70" s="3"/>
@@ -2896,7 +2896,7 @@
     </row>
     <row r="71" spans="1:12" ht="16">
       <c r="A71" s="2"/>
-      <c r="B71" s="22"/>
+      <c r="B71" s="31"/>
       <c r="C71" s="23"/>
       <c r="D71" s="2"/>
       <c r="E71" s="3"/>
@@ -2910,7 +2910,7 @@
     </row>
     <row r="72" spans="1:12" ht="16">
       <c r="A72" s="2"/>
-      <c r="B72" s="22"/>
+      <c r="B72" s="31"/>
       <c r="C72" s="23"/>
       <c r="D72" s="2"/>
       <c r="E72" s="3"/>
@@ -2924,7 +2924,7 @@
     </row>
     <row r="73" spans="1:12" ht="16">
       <c r="A73" s="2"/>
-      <c r="B73" s="22"/>
+      <c r="B73" s="31"/>
       <c r="C73" s="23"/>
       <c r="D73" s="2"/>
       <c r="E73" s="3"/>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="74" spans="1:12" ht="16">
       <c r="A74" s="2"/>
-      <c r="B74" s="22"/>
+      <c r="B74" s="31"/>
       <c r="C74" s="23"/>
       <c r="D74" s="2"/>
       <c r="E74" s="3"/>
@@ -2952,7 +2952,7 @@
     </row>
     <row r="75" spans="1:12" ht="16">
       <c r="A75" s="2"/>
-      <c r="B75" s="22"/>
+      <c r="B75" s="31"/>
       <c r="C75" s="23"/>
       <c r="D75" s="2"/>
       <c r="E75" s="3"/>
@@ -2966,7 +2966,7 @@
     </row>
     <row r="76" spans="1:12" ht="16">
       <c r="A76" s="2"/>
-      <c r="B76" s="22"/>
+      <c r="B76" s="31"/>
       <c r="C76" s="23"/>
       <c r="D76" s="2"/>
       <c r="E76" s="3"/>
@@ -2980,7 +2980,7 @@
     </row>
     <row r="77" spans="1:12" ht="16">
       <c r="A77" s="2"/>
-      <c r="B77" s="22"/>
+      <c r="B77" s="31"/>
       <c r="C77" s="23"/>
       <c r="D77" s="2"/>
       <c r="E77" s="3"/>
@@ -2994,7 +2994,7 @@
     </row>
     <row r="78" spans="1:12" ht="16">
       <c r="A78" s="2"/>
-      <c r="B78" s="22"/>
+      <c r="B78" s="31"/>
       <c r="C78" s="23"/>
       <c r="D78" s="2"/>
       <c r="E78" s="3"/>
@@ -3008,7 +3008,7 @@
     </row>
     <row r="79" spans="1:12" ht="16">
       <c r="A79" s="2"/>
-      <c r="B79" s="22"/>
+      <c r="B79" s="31"/>
       <c r="C79" s="23"/>
       <c r="D79" s="2"/>
       <c r="E79" s="3"/>
@@ -3022,7 +3022,7 @@
     </row>
     <row r="80" spans="1:12" ht="16">
       <c r="A80" s="2"/>
-      <c r="B80" s="22"/>
+      <c r="B80" s="31"/>
       <c r="C80" s="23"/>
       <c r="D80" s="2"/>
       <c r="E80" s="3"/>
@@ -3036,7 +3036,7 @@
     </row>
     <row r="81" spans="1:12" ht="16">
       <c r="A81" s="2"/>
-      <c r="B81" s="22"/>
+      <c r="B81" s="31"/>
       <c r="C81" s="23"/>
       <c r="D81" s="2"/>
       <c r="E81" s="3"/>
@@ -3050,7 +3050,7 @@
     </row>
     <row r="82" spans="1:12" ht="16">
       <c r="A82" s="2"/>
-      <c r="B82" s="22"/>
+      <c r="B82" s="31"/>
       <c r="C82" s="23"/>
       <c r="D82" s="2"/>
       <c r="E82" s="3"/>
@@ -3064,7 +3064,7 @@
     </row>
     <row r="83" spans="1:12" ht="16">
       <c r="A83" s="2"/>
-      <c r="B83" s="22"/>
+      <c r="B83" s="31"/>
       <c r="C83" s="23"/>
       <c r="D83" s="2"/>
       <c r="E83" s="3"/>
@@ -3078,7 +3078,7 @@
     </row>
     <row r="84" spans="1:12" ht="16">
       <c r="A84" s="2"/>
-      <c r="B84" s="22"/>
+      <c r="B84" s="31"/>
       <c r="C84" s="23"/>
       <c r="D84" s="2"/>
       <c r="E84" s="3"/>
@@ -3092,7 +3092,7 @@
     </row>
     <row r="85" spans="1:12" ht="16">
       <c r="A85" s="2"/>
-      <c r="B85" s="22"/>
+      <c r="B85" s="31"/>
       <c r="C85" s="23"/>
       <c r="D85" s="2"/>
       <c r="E85" s="3"/>
@@ -3106,26 +3106,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:G2"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A66:G66"/>
-    <mergeCell ref="D67:G67"/>
-    <mergeCell ref="D68:G68"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="B80:C80"/>
     <mergeCell ref="B74:C74"/>
@@ -3133,6 +3113,26 @@
     <mergeCell ref="B76:C76"/>
     <mergeCell ref="B77:C77"/>
     <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="D67:G67"/>
+    <mergeCell ref="D68:G68"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="A6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="A7:Z7">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">

</xml_diff>

<commit_message>
Hoan thien co ban cac chuc nang
</commit_message>
<xml_diff>
--- a/phan_giao.xlsx
+++ b/phan_giao.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pxvanhanh/TPM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6FAE902-A9F2-BE4D-AF32-F11952D8E30C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DF7F09-DA84-9741-BF0C-1866A3963E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PHÂN GIAO" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -38,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="162">
   <si>
     <t>CÔNG TY THỦY ĐIỆN BẢN VẼ
  PHÂN XƯỞNG VẬN HÀNH</t>
@@ -521,28 +534,22 @@
     <t>Đinh Anh Dũng</t>
   </si>
   <si>
-    <t>Trần Xuân Dức</t>
-  </si>
-  <si>
-    <t>Trần Xuân Dồng</t>
-  </si>
-  <si>
-    <t>Dậu Xuân Trung</t>
-  </si>
-  <si>
-    <t>Lê Dình Dũng</t>
-  </si>
-  <si>
-    <t>Lê Dình Long</t>
-  </si>
-  <si>
-    <t>Dào Duy Tùng</t>
-  </si>
-  <si>
-    <t>Nguyễn Dăng Kiên</t>
-  </si>
-  <si>
-    <t>Dương Dăng Tiến</t>
+    <t>Trần Xuân Đức</t>
+  </si>
+  <si>
+    <t>Trần Xuân Đồng</t>
+  </si>
+  <si>
+    <t>Đậu Xuân Trung</t>
+  </si>
+  <si>
+    <t>Lê Đình Dũng</t>
+  </si>
+  <si>
+    <t>Đào Duy Tùng</t>
+  </si>
+  <si>
+    <t>Dương Đăng Tiến</t>
   </si>
 </sst>
 </file>
@@ -789,19 +796,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -814,8 +812,17 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1069,11 +1076,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="16">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="23"/>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="28" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="23"/>
@@ -1105,7 +1112,7 @@
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="29" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="23"/>
@@ -1134,7 +1141,7 @@
     </row>
     <row r="5" spans="1:26" ht="17">
       <c r="A5" s="1"/>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="30" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="23"/>
@@ -1149,7 +1156,7 @@
       <c r="L5" s="4"/>
     </row>
     <row r="6" spans="1:26" ht="55.5" customHeight="1">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="31" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="23"/>
@@ -1416,7 +1423,7 @@
         <v>25</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>38</v>
@@ -1444,7 +1451,7 @@
         <v>25</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>38</v>
@@ -1528,7 +1535,7 @@
         <v>25</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>48</v>
@@ -1643,7 +1650,7 @@
         <v>52</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="G23" s="21">
         <v>1</v>
@@ -1671,7 +1678,7 @@
         <v>52</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="G24" s="21">
         <v>1</v>
@@ -1838,7 +1845,7 @@
       <c r="E30" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="F30" s="17" t="s">
+      <c r="F30" s="20" t="s">
         <v>156</v>
       </c>
       <c r="G30" s="21">
@@ -1866,7 +1873,7 @@
       <c r="E31" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="F31" s="17" t="s">
+      <c r="F31" s="20" t="s">
         <v>156</v>
       </c>
       <c r="G31" s="21">
@@ -1892,7 +1899,7 @@
         <v>51</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>160</v>
+        <v>77</v>
       </c>
       <c r="F32" s="16" t="s">
         <v>16</v>
@@ -1919,7 +1926,7 @@
       <c r="D33" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E33" s="20" t="s">
+      <c r="E33" s="17" t="s">
         <v>158</v>
       </c>
       <c r="F33" s="17" t="s">
@@ -2088,7 +2095,7 @@
         <v>74</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F39" s="20" t="s">
         <v>55</v>
@@ -2116,7 +2123,7 @@
         <v>74</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F40" s="20" t="s">
         <v>52</v>
@@ -2175,7 +2182,7 @@
         <v>100</v>
       </c>
       <c r="F42" s="20" t="s">
-        <v>160</v>
+        <v>77</v>
       </c>
       <c r="G42" s="21">
         <v>3</v>
@@ -2203,7 +2210,7 @@
         <v>105</v>
       </c>
       <c r="F43" s="20" t="s">
-        <v>160</v>
+        <v>77</v>
       </c>
       <c r="G43" s="21">
         <v>3</v>
@@ -2454,7 +2461,7 @@
       <c r="E52" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="F52" s="20" t="s">
+      <c r="F52" s="17" t="s">
         <v>158</v>
       </c>
       <c r="G52" s="21">
@@ -2538,7 +2545,7 @@
       <c r="E55" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="F55" s="20" t="s">
+      <c r="F55" s="17" t="s">
         <v>158</v>
       </c>
       <c r="G55" s="21">
@@ -2564,7 +2571,7 @@
         <v>74</v>
       </c>
       <c r="E56" s="20" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F56" s="17" t="s">
         <v>52</v>
@@ -2620,10 +2627,10 @@
         <v>74</v>
       </c>
       <c r="E58" s="20" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F58" s="20" t="s">
-        <v>160</v>
+        <v>77</v>
       </c>
       <c r="G58" s="21">
         <v>4</v>
@@ -2676,7 +2683,7 @@
         <v>74</v>
       </c>
       <c r="E60" s="20" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F60" s="17" t="s">
         <v>43</v>
@@ -2707,7 +2714,7 @@
         <v>84</v>
       </c>
       <c r="F61" s="17" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="G61" s="21">
         <v>4</v>
@@ -2735,7 +2742,7 @@
         <v>84</v>
       </c>
       <c r="F62" s="17" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="G62" s="21">
         <v>1</v>
@@ -2760,7 +2767,7 @@
         <v>74</v>
       </c>
       <c r="E63" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F63" s="17" t="s">
         <v>26</v>
@@ -2788,7 +2795,7 @@
         <v>74</v>
       </c>
       <c r="E64" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F64" s="20" t="s">
         <v>156</v>
@@ -2817,7 +2824,7 @@
       <c r="L65" s="3"/>
     </row>
     <row r="66" spans="1:12" ht="186.75" customHeight="1">
-      <c r="A66" s="27" t="s">
+      <c r="A66" s="24" t="s">
         <v>152</v>
       </c>
       <c r="B66" s="23"/>
@@ -2833,12 +2840,12 @@
       <c r="L66" s="3"/>
     </row>
     <row r="67" spans="1:12" ht="16">
-      <c r="A67" s="30" t="s">
+      <c r="A67" s="27" t="s">
         <v>153</v>
       </c>
       <c r="B67" s="23"/>
       <c r="C67" s="23"/>
-      <c r="D67" s="28" t="s">
+      <c r="D67" s="25" t="s">
         <v>154</v>
       </c>
       <c r="E67" s="23"/>
@@ -2851,10 +2858,10 @@
       <c r="L67" s="4"/>
     </row>
     <row r="68" spans="1:12" ht="16">
-      <c r="A68" s="31"/>
+      <c r="A68" s="22"/>
       <c r="B68" s="23"/>
       <c r="C68" s="23"/>
-      <c r="D68" s="29" t="s">
+      <c r="D68" s="26" t="s">
         <v>155</v>
       </c>
       <c r="E68" s="23"/>
@@ -2868,7 +2875,7 @@
     </row>
     <row r="69" spans="1:12" ht="16">
       <c r="A69" s="2"/>
-      <c r="B69" s="31"/>
+      <c r="B69" s="22"/>
       <c r="C69" s="23"/>
       <c r="D69" s="2"/>
       <c r="E69" s="3"/>
@@ -2882,7 +2889,7 @@
     </row>
     <row r="70" spans="1:12" ht="16">
       <c r="A70" s="2"/>
-      <c r="B70" s="31"/>
+      <c r="B70" s="22"/>
       <c r="C70" s="23"/>
       <c r="D70" s="2"/>
       <c r="E70" s="3"/>
@@ -2896,7 +2903,7 @@
     </row>
     <row r="71" spans="1:12" ht="16">
       <c r="A71" s="2"/>
-      <c r="B71" s="31"/>
+      <c r="B71" s="22"/>
       <c r="C71" s="23"/>
       <c r="D71" s="2"/>
       <c r="E71" s="3"/>
@@ -2910,7 +2917,7 @@
     </row>
     <row r="72" spans="1:12" ht="16">
       <c r="A72" s="2"/>
-      <c r="B72" s="31"/>
+      <c r="B72" s="22"/>
       <c r="C72" s="23"/>
       <c r="D72" s="2"/>
       <c r="E72" s="3"/>
@@ -2924,7 +2931,7 @@
     </row>
     <row r="73" spans="1:12" ht="16">
       <c r="A73" s="2"/>
-      <c r="B73" s="31"/>
+      <c r="B73" s="22"/>
       <c r="C73" s="23"/>
       <c r="D73" s="2"/>
       <c r="E73" s="3"/>
@@ -2938,7 +2945,7 @@
     </row>
     <row r="74" spans="1:12" ht="16">
       <c r="A74" s="2"/>
-      <c r="B74" s="31"/>
+      <c r="B74" s="22"/>
       <c r="C74" s="23"/>
       <c r="D74" s="2"/>
       <c r="E74" s="3"/>
@@ -2952,7 +2959,7 @@
     </row>
     <row r="75" spans="1:12" ht="16">
       <c r="A75" s="2"/>
-      <c r="B75" s="31"/>
+      <c r="B75" s="22"/>
       <c r="C75" s="23"/>
       <c r="D75" s="2"/>
       <c r="E75" s="3"/>
@@ -2966,7 +2973,7 @@
     </row>
     <row r="76" spans="1:12" ht="16">
       <c r="A76" s="2"/>
-      <c r="B76" s="31"/>
+      <c r="B76" s="22"/>
       <c r="C76" s="23"/>
       <c r="D76" s="2"/>
       <c r="E76" s="3"/>
@@ -2980,7 +2987,7 @@
     </row>
     <row r="77" spans="1:12" ht="16">
       <c r="A77" s="2"/>
-      <c r="B77" s="31"/>
+      <c r="B77" s="22"/>
       <c r="C77" s="23"/>
       <c r="D77" s="2"/>
       <c r="E77" s="3"/>
@@ -2994,7 +3001,7 @@
     </row>
     <row r="78" spans="1:12" ht="16">
       <c r="A78" s="2"/>
-      <c r="B78" s="31"/>
+      <c r="B78" s="22"/>
       <c r="C78" s="23"/>
       <c r="D78" s="2"/>
       <c r="E78" s="3"/>
@@ -3008,7 +3015,7 @@
     </row>
     <row r="79" spans="1:12" ht="16">
       <c r="A79" s="2"/>
-      <c r="B79" s="31"/>
+      <c r="B79" s="22"/>
       <c r="C79" s="23"/>
       <c r="D79" s="2"/>
       <c r="E79" s="3"/>
@@ -3022,7 +3029,7 @@
     </row>
     <row r="80" spans="1:12" ht="16">
       <c r="A80" s="2"/>
-      <c r="B80" s="31"/>
+      <c r="B80" s="22"/>
       <c r="C80" s="23"/>
       <c r="D80" s="2"/>
       <c r="E80" s="3"/>
@@ -3036,7 +3043,7 @@
     </row>
     <row r="81" spans="1:12" ht="16">
       <c r="A81" s="2"/>
-      <c r="B81" s="31"/>
+      <c r="B81" s="22"/>
       <c r="C81" s="23"/>
       <c r="D81" s="2"/>
       <c r="E81" s="3"/>
@@ -3050,7 +3057,7 @@
     </row>
     <row r="82" spans="1:12" ht="16">
       <c r="A82" s="2"/>
-      <c r="B82" s="31"/>
+      <c r="B82" s="22"/>
       <c r="C82" s="23"/>
       <c r="D82" s="2"/>
       <c r="E82" s="3"/>
@@ -3064,7 +3071,7 @@
     </row>
     <row r="83" spans="1:12" ht="16">
       <c r="A83" s="2"/>
-      <c r="B83" s="31"/>
+      <c r="B83" s="22"/>
       <c r="C83" s="23"/>
       <c r="D83" s="2"/>
       <c r="E83" s="3"/>
@@ -3078,7 +3085,7 @@
     </row>
     <row r="84" spans="1:12" ht="16">
       <c r="A84" s="2"/>
-      <c r="B84" s="31"/>
+      <c r="B84" s="22"/>
       <c r="C84" s="23"/>
       <c r="D84" s="2"/>
       <c r="E84" s="3"/>
@@ -3092,7 +3099,7 @@
     </row>
     <row r="85" spans="1:12" ht="16">
       <c r="A85" s="2"/>
-      <c r="B85" s="31"/>
+      <c r="B85" s="22"/>
       <c r="C85" s="23"/>
       <c r="D85" s="2"/>
       <c r="E85" s="3"/>
@@ -3106,6 +3113,26 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="D67:G67"/>
+    <mergeCell ref="D68:G68"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="B80:C80"/>
     <mergeCell ref="B74:C74"/>
@@ -3113,26 +3140,6 @@
     <mergeCell ref="B76:C76"/>
     <mergeCell ref="B77:C77"/>
     <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="A66:G66"/>
-    <mergeCell ref="D67:G67"/>
-    <mergeCell ref="D68:G68"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:G2"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="A6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="A7:Z7">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">

</xml_diff>

<commit_message>
Ban hoan thien F3 phan tach database may local
</commit_message>
<xml_diff>
--- a/phan_giao.xlsx
+++ b/phan_giao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pxvanhanh/TPM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DF7F09-DA84-9741-BF0C-1866A3963E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03687A67-2CC0-8E46-A547-561AAD2FACFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="161">
   <si>
     <t>CÔNG TY THỦY ĐIỆN BẢN VẼ
  PHÂN XƯỞNG VẬN HÀNH</t>
@@ -541,9 +541,6 @@
   </si>
   <si>
     <t>Đậu Xuân Trung</t>
-  </si>
-  <si>
-    <t>Lê Đình Dũng</t>
   </si>
   <si>
     <t>Đào Duy Tùng</t>
@@ -796,10 +793,19 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -812,17 +818,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1076,11 +1073,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="16">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="23"/>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="22" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="23"/>
@@ -1112,7 +1109,7 @@
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="24" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="23"/>
@@ -1141,7 +1138,7 @@
     </row>
     <row r="5" spans="1:26" ht="17">
       <c r="A5" s="1"/>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="25" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="23"/>
@@ -1156,7 +1153,7 @@
       <c r="L5" s="4"/>
     </row>
     <row r="6" spans="1:26" ht="55.5" customHeight="1">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="26" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="23"/>
@@ -1815,7 +1812,7 @@
         <v>51</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F29" s="17" t="s">
         <v>26</v>
@@ -1843,7 +1840,7 @@
         <v>74</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F30" s="20" t="s">
         <v>156</v>
@@ -2014,7 +2011,7 @@
         <v>89</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G36" s="21">
         <v>5</v>
@@ -2042,7 +2039,7 @@
         <v>89</v>
       </c>
       <c r="F37" s="17" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G37" s="21">
         <v>5</v>
@@ -2095,7 +2092,7 @@
         <v>74</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F39" s="20" t="s">
         <v>55</v>
@@ -2123,7 +2120,7 @@
         <v>74</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F40" s="20" t="s">
         <v>52</v>
@@ -2322,7 +2319,7 @@
         <v>100</v>
       </c>
       <c r="F47" s="17" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G47" s="21">
         <v>3</v>
@@ -2571,7 +2568,7 @@
         <v>74</v>
       </c>
       <c r="E56" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F56" s="17" t="s">
         <v>52</v>
@@ -2627,7 +2624,7 @@
         <v>74</v>
       </c>
       <c r="E58" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F58" s="20" t="s">
         <v>77</v>
@@ -2683,7 +2680,7 @@
         <v>74</v>
       </c>
       <c r="E60" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F60" s="17" t="s">
         <v>43</v>
@@ -2767,7 +2764,7 @@
         <v>74</v>
       </c>
       <c r="E63" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F63" s="17" t="s">
         <v>26</v>
@@ -2795,7 +2792,7 @@
         <v>74</v>
       </c>
       <c r="E64" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F64" s="20" t="s">
         <v>156</v>
@@ -2824,7 +2821,7 @@
       <c r="L65" s="3"/>
     </row>
     <row r="66" spans="1:12" ht="186.75" customHeight="1">
-      <c r="A66" s="24" t="s">
+      <c r="A66" s="27" t="s">
         <v>152</v>
       </c>
       <c r="B66" s="23"/>
@@ -2840,12 +2837,12 @@
       <c r="L66" s="3"/>
     </row>
     <row r="67" spans="1:12" ht="16">
-      <c r="A67" s="27" t="s">
+      <c r="A67" s="30" t="s">
         <v>153</v>
       </c>
       <c r="B67" s="23"/>
       <c r="C67" s="23"/>
-      <c r="D67" s="25" t="s">
+      <c r="D67" s="28" t="s">
         <v>154</v>
       </c>
       <c r="E67" s="23"/>
@@ -2858,10 +2855,10 @@
       <c r="L67" s="4"/>
     </row>
     <row r="68" spans="1:12" ht="16">
-      <c r="A68" s="22"/>
+      <c r="A68" s="31"/>
       <c r="B68" s="23"/>
       <c r="C68" s="23"/>
-      <c r="D68" s="26" t="s">
+      <c r="D68" s="29" t="s">
         <v>155</v>
       </c>
       <c r="E68" s="23"/>
@@ -2875,7 +2872,7 @@
     </row>
     <row r="69" spans="1:12" ht="16">
       <c r="A69" s="2"/>
-      <c r="B69" s="22"/>
+      <c r="B69" s="31"/>
       <c r="C69" s="23"/>
       <c r="D69" s="2"/>
       <c r="E69" s="3"/>
@@ -2889,7 +2886,7 @@
     </row>
     <row r="70" spans="1:12" ht="16">
       <c r="A70" s="2"/>
-      <c r="B70" s="22"/>
+      <c r="B70" s="31"/>
       <c r="C70" s="23"/>
       <c r="D70" s="2"/>
       <c r="E70" s="3"/>
@@ -2903,7 +2900,7 @@
     </row>
     <row r="71" spans="1:12" ht="16">
       <c r="A71" s="2"/>
-      <c r="B71" s="22"/>
+      <c r="B71" s="31"/>
       <c r="C71" s="23"/>
       <c r="D71" s="2"/>
       <c r="E71" s="3"/>
@@ -2917,7 +2914,7 @@
     </row>
     <row r="72" spans="1:12" ht="16">
       <c r="A72" s="2"/>
-      <c r="B72" s="22"/>
+      <c r="B72" s="31"/>
       <c r="C72" s="23"/>
       <c r="D72" s="2"/>
       <c r="E72" s="3"/>
@@ -2931,7 +2928,7 @@
     </row>
     <row r="73" spans="1:12" ht="16">
       <c r="A73" s="2"/>
-      <c r="B73" s="22"/>
+      <c r="B73" s="31"/>
       <c r="C73" s="23"/>
       <c r="D73" s="2"/>
       <c r="E73" s="3"/>
@@ -2945,7 +2942,7 @@
     </row>
     <row r="74" spans="1:12" ht="16">
       <c r="A74" s="2"/>
-      <c r="B74" s="22"/>
+      <c r="B74" s="31"/>
       <c r="C74" s="23"/>
       <c r="D74" s="2"/>
       <c r="E74" s="3"/>
@@ -2959,7 +2956,7 @@
     </row>
     <row r="75" spans="1:12" ht="16">
       <c r="A75" s="2"/>
-      <c r="B75" s="22"/>
+      <c r="B75" s="31"/>
       <c r="C75" s="23"/>
       <c r="D75" s="2"/>
       <c r="E75" s="3"/>
@@ -2973,7 +2970,7 @@
     </row>
     <row r="76" spans="1:12" ht="16">
       <c r="A76" s="2"/>
-      <c r="B76" s="22"/>
+      <c r="B76" s="31"/>
       <c r="C76" s="23"/>
       <c r="D76" s="2"/>
       <c r="E76" s="3"/>
@@ -2987,7 +2984,7 @@
     </row>
     <row r="77" spans="1:12" ht="16">
       <c r="A77" s="2"/>
-      <c r="B77" s="22"/>
+      <c r="B77" s="31"/>
       <c r="C77" s="23"/>
       <c r="D77" s="2"/>
       <c r="E77" s="3"/>
@@ -3001,7 +2998,7 @@
     </row>
     <row r="78" spans="1:12" ht="16">
       <c r="A78" s="2"/>
-      <c r="B78" s="22"/>
+      <c r="B78" s="31"/>
       <c r="C78" s="23"/>
       <c r="D78" s="2"/>
       <c r="E78" s="3"/>
@@ -3015,7 +3012,7 @@
     </row>
     <row r="79" spans="1:12" ht="16">
       <c r="A79" s="2"/>
-      <c r="B79" s="22"/>
+      <c r="B79" s="31"/>
       <c r="C79" s="23"/>
       <c r="D79" s="2"/>
       <c r="E79" s="3"/>
@@ -3029,7 +3026,7 @@
     </row>
     <row r="80" spans="1:12" ht="16">
       <c r="A80" s="2"/>
-      <c r="B80" s="22"/>
+      <c r="B80" s="31"/>
       <c r="C80" s="23"/>
       <c r="D80" s="2"/>
       <c r="E80" s="3"/>
@@ -3043,7 +3040,7 @@
     </row>
     <row r="81" spans="1:12" ht="16">
       <c r="A81" s="2"/>
-      <c r="B81" s="22"/>
+      <c r="B81" s="31"/>
       <c r="C81" s="23"/>
       <c r="D81" s="2"/>
       <c r="E81" s="3"/>
@@ -3057,7 +3054,7 @@
     </row>
     <row r="82" spans="1:12" ht="16">
       <c r="A82" s="2"/>
-      <c r="B82" s="22"/>
+      <c r="B82" s="31"/>
       <c r="C82" s="23"/>
       <c r="D82" s="2"/>
       <c r="E82" s="3"/>
@@ -3071,7 +3068,7 @@
     </row>
     <row r="83" spans="1:12" ht="16">
       <c r="A83" s="2"/>
-      <c r="B83" s="22"/>
+      <c r="B83" s="31"/>
       <c r="C83" s="23"/>
       <c r="D83" s="2"/>
       <c r="E83" s="3"/>
@@ -3085,7 +3082,7 @@
     </row>
     <row r="84" spans="1:12" ht="16">
       <c r="A84" s="2"/>
-      <c r="B84" s="22"/>
+      <c r="B84" s="31"/>
       <c r="C84" s="23"/>
       <c r="D84" s="2"/>
       <c r="E84" s="3"/>
@@ -3099,7 +3096,7 @@
     </row>
     <row r="85" spans="1:12" ht="16">
       <c r="A85" s="2"/>
-      <c r="B85" s="22"/>
+      <c r="B85" s="31"/>
       <c r="C85" s="23"/>
       <c r="D85" s="2"/>
       <c r="E85" s="3"/>
@@ -3113,26 +3110,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:G2"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A66:G66"/>
-    <mergeCell ref="D67:G67"/>
-    <mergeCell ref="D68:G68"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="B80:C80"/>
     <mergeCell ref="B74:C74"/>
@@ -3140,6 +3117,26 @@
     <mergeCell ref="B76:C76"/>
     <mergeCell ref="B77:C77"/>
     <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="D67:G67"/>
+    <mergeCell ref="D68:G68"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="A6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="A7:Z7">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">

</xml_diff>

<commit_message>
update: phan cong moi
</commit_message>
<xml_diff>
--- a/phan_giao.xlsx
+++ b/phan_giao.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pxvanhanh/TPM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03687A67-2CC0-8E46-A547-561AAD2FACFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30669321-2531-1748-89AC-F74A15333BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PHÂN GIAO" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="160">
   <si>
     <t>CÔNG TY THỦY ĐIỆN BẢN VẼ
  PHÂN XƯỞNG VẬN HÀNH</t>
@@ -64,9 +64,6 @@
     <t>Số: /PXVH</t>
   </si>
   <si>
-    <t>Bản Vẽ, ngày 01 tháng 02 năm 2026</t>
-  </si>
-  <si>
     <t>PHÂN CÔNG THỰC HIỆN ĐÁNH GIÁ CÁC BIỂU MẪU BẢO TRÌ TỰ QUẢN
  (NĂM 2026)</t>
   </si>
@@ -211,9 +208,6 @@
     <t>BM.P4.15.13</t>
   </si>
   <si>
-    <t>Trực chính</t>
-  </si>
-  <si>
     <t>Trần Thế Anh</t>
   </si>
   <si>
@@ -278,9 +272,6 @@
   </si>
   <si>
     <t>BM.P4.15.23</t>
-  </si>
-  <si>
-    <t>Trực phụ</t>
   </si>
   <si>
     <t>HỆ THỐNG TỰ DÙNG 1 CHIỀU TRẠM</t>
@@ -526,27 +517,33 @@
  - Lưu PXVH</t>
   </si>
   <si>
-    <t xml:space="preserve">KT QUẢN ĐỐC
+    <t>Đinh Anh Dũng</t>
+  </si>
+  <si>
+    <t>Trần Xuân Đức</t>
+  </si>
+  <si>
+    <t>Trần Xuân Đồng</t>
+  </si>
+  <si>
+    <t>Đậu Xuân Trung</t>
+  </si>
+  <si>
+    <t>Đào Duy Tùng</t>
+  </si>
+  <si>
+    <t>Dương Đăng Tiến</t>
+  </si>
+  <si>
+    <t>Bản Vẽ, ngày 01 tháng 08 năm 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUẢN ĐỐC
  PHÓ QUẢN ĐỐC
 </t>
   </si>
   <si>
-    <t>Đinh Anh Dũng</t>
-  </si>
-  <si>
-    <t>Trần Xuân Đức</t>
-  </si>
-  <si>
-    <t>Trần Xuân Đồng</t>
-  </si>
-  <si>
-    <t>Đậu Xuân Trung</t>
-  </si>
-  <si>
-    <t>Đào Duy Tùng</t>
-  </si>
-  <si>
-    <t>Dương Đăng Tiến</t>
+    <t>VHV</t>
   </si>
 </sst>
 </file>
@@ -600,11 +597,6 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="&quot;Times New Roman&quot;"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="&quot;Times New Roman&quot;"/>
@@ -624,6 +616,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -639,7 +637,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -734,11 +732,44 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -778,25 +809,28 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -806,21 +840,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1059,7 +1091,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Z85"/>
@@ -1076,14 +1108,14 @@
       <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
+      <c r="B1" s="18"/>
       <c r="C1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
       <c r="H1" s="2"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -1091,13 +1123,13 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:26" ht="16">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
       <c r="H2" s="2"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
@@ -1109,13 +1141,13 @@
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
+      <c r="C3" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
       <c r="H3" s="2"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -1138,30 +1170,30 @@
     </row>
     <row r="5" spans="1:26" ht="17">
       <c r="A5" s="1"/>
-      <c r="B5" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
+      <c r="B5" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
     </row>
     <row r="6" spans="1:26" ht="55.5" customHeight="1">
-      <c r="A6" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
+      <c r="A6" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
       <c r="H6" s="5"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
@@ -1170,25 +1202,25 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="D7" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="F7" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>11</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>12</v>
       </c>
       <c r="H7" s="11"/>
       <c r="I7" s="11"/>
@@ -1215,21 +1247,21 @@
         <v>1</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="D8" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="E8" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="F8" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" s="18">
+      <c r="G8" s="15">
         <v>2</v>
       </c>
       <c r="H8" s="2"/>
@@ -1243,21 +1275,21 @@
         <v>2</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="21">
+      <c r="D9" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="16">
         <v>2</v>
       </c>
       <c r="H9" s="2"/>
@@ -1271,21 +1303,21 @@
         <v>3</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="21">
+      <c r="D10" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="16">
         <v>2</v>
       </c>
       <c r="H10" s="2"/>
@@ -1299,21 +1331,21 @@
         <v>4</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="D11" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="21">
+      <c r="G11" s="16">
         <v>3</v>
       </c>
       <c r="H11" s="2"/>
@@ -1327,21 +1359,21 @@
         <v>5</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="20" t="s">
+      <c r="D12" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="F12" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="21">
+      <c r="G12" s="16">
         <v>3</v>
       </c>
       <c r="H12" s="2"/>
@@ -1355,21 +1387,21 @@
         <v>6</v>
       </c>
       <c r="B13" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="G13" s="21">
+      <c r="D13" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="16">
         <v>1</v>
       </c>
       <c r="H13" s="2"/>
@@ -1383,21 +1415,21 @@
         <v>7</v>
       </c>
       <c r="B14" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="F14" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="G14" s="21">
+      <c r="D14" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="16">
         <v>1</v>
       </c>
       <c r="H14" s="2"/>
@@ -1411,21 +1443,21 @@
         <v>8</v>
       </c>
       <c r="B15" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="F15" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="G15" s="21">
+      <c r="D15" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="16">
         <v>5</v>
       </c>
       <c r="H15" s="2"/>
@@ -1439,21 +1471,21 @@
         <v>9</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="G16" s="21">
+      <c r="D16" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="16">
         <v>5</v>
       </c>
       <c r="H16" s="2"/>
@@ -1467,21 +1499,21 @@
         <v>10</v>
       </c>
       <c r="B17" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="D17" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="F17" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="F17" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="G17" s="21">
+      <c r="G17" s="16">
         <v>2</v>
       </c>
       <c r="H17" s="2"/>
@@ -1495,21 +1527,21 @@
         <v>11</v>
       </c>
       <c r="B18" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="F18" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="G18" s="21">
+      <c r="D18" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="F18" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="G18" s="16">
         <v>2</v>
       </c>
       <c r="H18" s="2"/>
@@ -1523,21 +1555,21 @@
         <v>12</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="F19" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="G19" s="21">
+      <c r="D19" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="16">
         <v>2</v>
       </c>
       <c r="H19" s="2"/>
@@ -1551,21 +1583,21 @@
         <v>13</v>
       </c>
       <c r="B20" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E20" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="F20" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G20" s="21">
+      <c r="D20" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E20" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="F20" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="16">
         <v>2</v>
       </c>
       <c r="H20" s="2"/>
@@ -1579,21 +1611,21 @@
         <v>14</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="F21" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="G21" s="21">
+      <c r="C21" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E21" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21" s="16">
         <v>6</v>
       </c>
       <c r="H21" s="2"/>
@@ -1607,21 +1639,21 @@
         <v>15</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D22" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="F22" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="G22" s="21">
+      <c r="D22" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E22" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="G22" s="16">
         <v>6</v>
       </c>
       <c r="H22" s="2"/>
@@ -1635,21 +1667,21 @@
         <v>16</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E23" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="F23" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="G23" s="21">
+        <v>56</v>
+      </c>
+      <c r="C23" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E23" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="F23" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="G23" s="16">
         <v>1</v>
       </c>
       <c r="H23" s="2"/>
@@ -1663,21 +1695,21 @@
         <v>17</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E24" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="G24" s="21">
+        <v>58</v>
+      </c>
+      <c r="C24" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E24" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="G24" s="16">
         <v>1</v>
       </c>
       <c r="H24" s="2"/>
@@ -1691,21 +1723,21 @@
         <v>18</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E25" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="F25" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="G25" s="21">
+        <v>60</v>
+      </c>
+      <c r="C25" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E25" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="F25" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="G25" s="16">
         <v>4</v>
       </c>
       <c r="H25" s="2"/>
@@ -1719,21 +1751,21 @@
         <v>19</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E26" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="F26" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="G26" s="21">
+        <v>62</v>
+      </c>
+      <c r="C26" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E26" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="F26" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" s="16">
         <v>4</v>
       </c>
       <c r="H26" s="2"/>
@@ -1747,21 +1779,21 @@
         <v>20</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="D27" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E27" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="F27" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G27" s="21">
+        <v>64</v>
+      </c>
+      <c r="C27" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E27" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="F27" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="G27" s="16">
         <v>2</v>
       </c>
       <c r="H27" s="2"/>
@@ -1775,21 +1807,21 @@
         <v>21</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="D28" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E28" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="F28" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="G28" s="21">
+        <v>66</v>
+      </c>
+      <c r="C28" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E28" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="F28" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="16">
         <v>3</v>
       </c>
       <c r="H28" s="2"/>
@@ -1803,21 +1835,21 @@
         <v>22</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="C29" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="D29" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="F29" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="G29" s="21">
+        <v>68</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E29" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="F29" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="G29" s="16">
         <v>3</v>
       </c>
       <c r="H29" s="2"/>
@@ -1831,21 +1863,21 @@
         <v>23</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="D30" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="F30" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="G30" s="21">
+        <v>70</v>
+      </c>
+      <c r="C30" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="D30" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E30" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="F30" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="G30" s="16">
         <v>5</v>
       </c>
       <c r="H30" s="2"/>
@@ -1859,21 +1891,21 @@
         <v>24</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C31" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E31" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="F31" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="G31" s="21">
+        <v>72</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="D31" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E31" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="F31" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" s="16">
         <v>1</v>
       </c>
       <c r="H31" s="2"/>
@@ -1887,21 +1919,21 @@
         <v>25</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="C32" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="D32" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E32" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="F32" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="G32" s="21">
+        <v>75</v>
+      </c>
+      <c r="C32" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E32" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="F32" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="G32" s="16">
         <v>5</v>
       </c>
       <c r="H32" s="2"/>
@@ -1915,21 +1947,21 @@
         <v>26</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="C33" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="D33" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="E33" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="F33" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="G33" s="21">
+        <v>77</v>
+      </c>
+      <c r="C33" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E33" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="F33" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="G33" s="16">
         <v>5</v>
       </c>
       <c r="H33" s="2"/>
@@ -1943,21 +1975,21 @@
         <v>27</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="C34" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="D34" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E34" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="F34" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="G34" s="21">
+        <v>79</v>
+      </c>
+      <c r="C34" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E34" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="F34" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34" s="16">
         <v>2</v>
       </c>
       <c r="H34" s="2"/>
@@ -1971,21 +2003,21 @@
         <v>28</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C35" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="D35" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E35" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="F35" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="E35" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="F35" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="G35" s="21">
+      <c r="G35" s="16">
         <v>2</v>
       </c>
       <c r="H35" s="2"/>
@@ -1999,21 +2031,21 @@
         <v>29</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C36" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="D36" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E36" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="F36" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="G36" s="21">
+        <v>84</v>
+      </c>
+      <c r="C36" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D36" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E36" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="F36" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="G36" s="16">
         <v>5</v>
       </c>
       <c r="H36" s="2"/>
@@ -2027,21 +2059,21 @@
         <v>30</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C37" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="D37" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E37" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="F37" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="G37" s="21">
+        <v>87</v>
+      </c>
+      <c r="C37" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D37" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E37" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="F37" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="G37" s="16">
         <v>5</v>
       </c>
       <c r="H37" s="2"/>
@@ -2055,21 +2087,21 @@
         <v>31</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C38" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="D38" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E38" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="F38" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="G38" s="21">
+      <c r="C38" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="D38" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E38" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="F38" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="G38" s="16">
         <v>4</v>
       </c>
       <c r="H38" s="2"/>
@@ -2083,21 +2115,21 @@
         <v>32</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C39" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="D39" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E39" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="F39" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="G39" s="21">
+        <v>91</v>
+      </c>
+      <c r="C39" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E39" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="F39" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="G39" s="16">
         <v>4</v>
       </c>
       <c r="H39" s="2"/>
@@ -2111,21 +2143,21 @@
         <v>33</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C40" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="D40" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="C40" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="D40" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E40" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="F40" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="E40" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="F40" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="G40" s="21">
+      <c r="G40" s="16">
         <v>1</v>
       </c>
       <c r="H40" s="2"/>
@@ -2139,21 +2171,21 @@
         <v>34</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="C41" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="D41" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E41" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="F41" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="G41" s="21">
+        <v>95</v>
+      </c>
+      <c r="C41" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="D41" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E41" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="F41" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="G41" s="16">
         <v>1</v>
       </c>
       <c r="H41" s="2"/>
@@ -2167,21 +2199,21 @@
         <v>35</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="C42" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="D42" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E42" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="F42" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="G42" s="21">
+        <v>98</v>
+      </c>
+      <c r="C42" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="D42" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E42" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="F42" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="G42" s="16">
         <v>3</v>
       </c>
       <c r="H42" s="2"/>
@@ -2195,21 +2227,21 @@
         <v>36</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C43" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="D43" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E43" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="F43" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="G43" s="21">
+        <v>100</v>
+      </c>
+      <c r="C43" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="D43" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E43" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="F43" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="G43" s="16">
         <v>3</v>
       </c>
       <c r="H43" s="2"/>
@@ -2223,21 +2255,21 @@
         <v>37</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C44" s="19" t="s">
-        <v>107</v>
-      </c>
-      <c r="D44" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E44" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="F44" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="G44" s="21">
+        <v>103</v>
+      </c>
+      <c r="C44" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D44" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E44" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="F44" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="G44" s="16">
         <v>2</v>
       </c>
       <c r="H44" s="2"/>
@@ -2251,21 +2283,21 @@
         <v>38</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="D45" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E45" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="F45" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="G45" s="21">
+        <v>106</v>
+      </c>
+      <c r="C45" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D45" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E45" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="F45" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="G45" s="16">
         <v>2</v>
       </c>
       <c r="H45" s="2"/>
@@ -2279,21 +2311,21 @@
         <v>39</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="C46" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="D46" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E46" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="F46" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G46" s="21">
+      <c r="C46" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="D46" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E46" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="F46" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="G46" s="16">
         <v>3</v>
       </c>
       <c r="H46" s="2"/>
@@ -2307,21 +2339,21 @@
         <v>40</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="C47" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="D47" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E47" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="F47" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="G47" s="21">
+        <v>110</v>
+      </c>
+      <c r="C47" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="D47" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E47" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="F47" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="G47" s="16">
         <v>3</v>
       </c>
       <c r="H47" s="2"/>
@@ -2335,21 +2367,21 @@
         <v>41</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="C48" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="D48" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C48" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="D48" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E48" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="F48" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="E48" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="F48" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="G48" s="21">
+      <c r="G48" s="16">
         <v>6</v>
       </c>
       <c r="H48" s="2"/>
@@ -2363,21 +2395,21 @@
         <v>42</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="D49" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C49" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="D49" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E49" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="F49" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="E49" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="F49" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="G49" s="21">
+      <c r="G49" s="16">
         <v>6</v>
       </c>
       <c r="H49" s="2"/>
@@ -2391,21 +2423,21 @@
         <v>43</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="C50" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="D50" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E50" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="F50" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="G50" s="21">
+        <v>117</v>
+      </c>
+      <c r="C50" s="28" t="s">
+        <v>118</v>
+      </c>
+      <c r="D50" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E50" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="F50" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="G50" s="16">
         <v>1</v>
       </c>
       <c r="H50" s="2"/>
@@ -2419,21 +2451,21 @@
         <v>44</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="C51" s="19" t="s">
-        <v>124</v>
-      </c>
-      <c r="D51" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E51" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="F51" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="G51" s="21">
+        <v>120</v>
+      </c>
+      <c r="C51" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="D51" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E51" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="F51" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="G51" s="16">
         <v>1</v>
       </c>
       <c r="H51" s="2"/>
@@ -2447,21 +2479,21 @@
         <v>45</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="C52" s="19" t="s">
-        <v>126</v>
-      </c>
-      <c r="D52" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E52" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="F52" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="G52" s="21">
+        <v>122</v>
+      </c>
+      <c r="C52" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="D52" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E52" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="F52" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="G52" s="16">
         <v>3</v>
       </c>
       <c r="H52" s="2"/>
@@ -2475,21 +2507,21 @@
         <v>46</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="C53" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="D53" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E53" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="F53" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="G53" s="21">
+        <v>124</v>
+      </c>
+      <c r="C53" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="D53" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E53" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="F53" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="G53" s="16">
         <v>3</v>
       </c>
       <c r="H53" s="2"/>
@@ -2503,21 +2535,21 @@
         <v>47</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E54" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="F54" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G54" s="21">
+        <v>127</v>
+      </c>
+      <c r="C54" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="D54" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E54" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="F54" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="G54" s="16">
         <v>5</v>
       </c>
       <c r="H54" s="2"/>
@@ -2531,21 +2563,21 @@
         <v>48</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="C55" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="D55" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E55" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="F55" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="G55" s="21">
+      <c r="C55" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="D55" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E55" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="F55" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="G55" s="16">
         <v>5</v>
       </c>
       <c r="H55" s="2"/>
@@ -2559,21 +2591,21 @@
         <v>49</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="C56" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D56" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E56" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="F56" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="G56" s="21">
+        <v>131</v>
+      </c>
+      <c r="C56" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="D56" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E56" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="F56" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="G56" s="16">
         <v>2</v>
       </c>
       <c r="H56" s="2"/>
@@ -2587,21 +2619,21 @@
         <v>50</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="C57" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="D57" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E57" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="F57" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="G57" s="21">
+        <v>133</v>
+      </c>
+      <c r="C57" s="28" t="s">
+        <v>134</v>
+      </c>
+      <c r="D57" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E57" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="F57" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="G57" s="16">
         <v>1</v>
       </c>
       <c r="H57" s="2"/>
@@ -2615,21 +2647,21 @@
         <v>51</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="D58" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E58" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="F58" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="G58" s="21">
+        <v>135</v>
+      </c>
+      <c r="C58" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="D58" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E58" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="F58" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="G58" s="16">
         <v>4</v>
       </c>
       <c r="H58" s="2"/>
@@ -2643,21 +2675,21 @@
         <v>52</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="C59" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="D59" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E59" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="F59" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="G59" s="21">
+        <v>137</v>
+      </c>
+      <c r="C59" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="D59" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E59" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="F59" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="G59" s="16">
         <v>2</v>
       </c>
       <c r="H59" s="2"/>
@@ -2671,21 +2703,21 @@
         <v>53</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="C60" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="D60" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="C60" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="D60" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E60" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="F60" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="E60" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="F60" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="G60" s="21">
+      <c r="G60" s="16">
         <v>4</v>
       </c>
       <c r="H60" s="2"/>
@@ -2699,21 +2731,21 @@
         <v>54</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C61" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="D61" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E61" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="F61" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="G61" s="21">
+        <v>141</v>
+      </c>
+      <c r="C61" s="28" t="s">
+        <v>142</v>
+      </c>
+      <c r="D61" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E61" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="F61" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="G61" s="16">
         <v>4</v>
       </c>
       <c r="H61" s="2"/>
@@ -2727,21 +2759,21 @@
         <v>55</v>
       </c>
       <c r="B62" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="C62" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="D62" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E62" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="F62" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="G62" s="21">
+        <v>143</v>
+      </c>
+      <c r="C62" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="D62" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E62" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="F62" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="G62" s="16">
         <v>1</v>
       </c>
       <c r="H62" s="2"/>
@@ -2755,21 +2787,21 @@
         <v>56</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="C63" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="D63" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E63" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="F63" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="G63" s="21">
+        <v>145</v>
+      </c>
+      <c r="C63" s="28" t="s">
+        <v>146</v>
+      </c>
+      <c r="D63" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E63" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="F63" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="G63" s="16">
         <v>6</v>
       </c>
       <c r="H63" s="2"/>
@@ -2783,21 +2815,21 @@
         <v>57</v>
       </c>
       <c r="B64" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="C64" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="D64" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E64" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="F64" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="G64" s="21">
+        <v>147</v>
+      </c>
+      <c r="C64" s="28" t="s">
+        <v>148</v>
+      </c>
+      <c r="D64" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E64" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="F64" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="G64" s="16">
         <v>6</v>
       </c>
       <c r="H64" s="2"/>
@@ -2821,15 +2853,15 @@
       <c r="L65" s="3"/>
     </row>
     <row r="66" spans="1:12" ht="186.75" customHeight="1">
-      <c r="A66" s="27" t="s">
-        <v>152</v>
-      </c>
-      <c r="B66" s="23"/>
-      <c r="C66" s="23"/>
-      <c r="D66" s="23"/>
-      <c r="E66" s="23"/>
-      <c r="F66" s="23"/>
-      <c r="G66" s="23"/>
+      <c r="A66" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="B66" s="18"/>
+      <c r="C66" s="18"/>
+      <c r="D66" s="18"/>
+      <c r="E66" s="18"/>
+      <c r="F66" s="18"/>
+      <c r="G66" s="18"/>
       <c r="H66" s="2"/>
       <c r="I66" s="3"/>
       <c r="J66" s="3"/>
@@ -2837,17 +2869,17 @@
       <c r="L66" s="3"/>
     </row>
     <row r="67" spans="1:12" ht="16">
-      <c r="A67" s="30" t="s">
-        <v>153</v>
-      </c>
-      <c r="B67" s="23"/>
-      <c r="C67" s="23"/>
-      <c r="D67" s="28" t="s">
-        <v>154</v>
-      </c>
-      <c r="E67" s="23"/>
-      <c r="F67" s="23"/>
-      <c r="G67" s="23"/>
+      <c r="A67" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="B67" s="18"/>
+      <c r="C67" s="18"/>
+      <c r="D67" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="E67" s="18"/>
+      <c r="F67" s="18"/>
+      <c r="G67" s="18"/>
       <c r="H67" s="2"/>
       <c r="I67" s="3"/>
       <c r="J67" s="3"/>
@@ -2855,15 +2887,15 @@
       <c r="L67" s="4"/>
     </row>
     <row r="68" spans="1:12" ht="16">
-      <c r="A68" s="31"/>
-      <c r="B68" s="23"/>
-      <c r="C68" s="23"/>
-      <c r="D68" s="29" t="s">
-        <v>155</v>
-      </c>
-      <c r="E68" s="23"/>
-      <c r="F68" s="23"/>
-      <c r="G68" s="23"/>
+      <c r="A68" s="17"/>
+      <c r="B68" s="18"/>
+      <c r="C68" s="18"/>
+      <c r="D68" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="E68" s="18"/>
+      <c r="F68" s="18"/>
+      <c r="G68" s="18"/>
       <c r="H68" s="2"/>
       <c r="I68" s="3"/>
       <c r="J68" s="3"/>
@@ -2872,8 +2904,8 @@
     </row>
     <row r="69" spans="1:12" ht="16">
       <c r="A69" s="2"/>
-      <c r="B69" s="31"/>
-      <c r="C69" s="23"/>
+      <c r="B69" s="17"/>
+      <c r="C69" s="18"/>
       <c r="D69" s="2"/>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
@@ -2886,8 +2918,8 @@
     </row>
     <row r="70" spans="1:12" ht="16">
       <c r="A70" s="2"/>
-      <c r="B70" s="31"/>
-      <c r="C70" s="23"/>
+      <c r="B70" s="17"/>
+      <c r="C70" s="18"/>
       <c r="D70" s="2"/>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
@@ -2900,8 +2932,8 @@
     </row>
     <row r="71" spans="1:12" ht="16">
       <c r="A71" s="2"/>
-      <c r="B71" s="31"/>
-      <c r="C71" s="23"/>
+      <c r="B71" s="17"/>
+      <c r="C71" s="18"/>
       <c r="D71" s="2"/>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
@@ -2914,8 +2946,8 @@
     </row>
     <row r="72" spans="1:12" ht="16">
       <c r="A72" s="2"/>
-      <c r="B72" s="31"/>
-      <c r="C72" s="23"/>
+      <c r="B72" s="17"/>
+      <c r="C72" s="18"/>
       <c r="D72" s="2"/>
       <c r="E72" s="3"/>
       <c r="F72" s="4"/>
@@ -2928,8 +2960,8 @@
     </row>
     <row r="73" spans="1:12" ht="16">
       <c r="A73" s="2"/>
-      <c r="B73" s="31"/>
-      <c r="C73" s="23"/>
+      <c r="B73" s="17"/>
+      <c r="C73" s="18"/>
       <c r="D73" s="2"/>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
@@ -2942,8 +2974,8 @@
     </row>
     <row r="74" spans="1:12" ht="16">
       <c r="A74" s="2"/>
-      <c r="B74" s="31"/>
-      <c r="C74" s="23"/>
+      <c r="B74" s="17"/>
+      <c r="C74" s="18"/>
       <c r="D74" s="2"/>
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
@@ -2956,8 +2988,8 @@
     </row>
     <row r="75" spans="1:12" ht="16">
       <c r="A75" s="2"/>
-      <c r="B75" s="31"/>
-      <c r="C75" s="23"/>
+      <c r="B75" s="17"/>
+      <c r="C75" s="18"/>
       <c r="D75" s="2"/>
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
@@ -2970,8 +3002,8 @@
     </row>
     <row r="76" spans="1:12" ht="16">
       <c r="A76" s="2"/>
-      <c r="B76" s="31"/>
-      <c r="C76" s="23"/>
+      <c r="B76" s="17"/>
+      <c r="C76" s="18"/>
       <c r="D76" s="2"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
@@ -2984,8 +3016,8 @@
     </row>
     <row r="77" spans="1:12" ht="16">
       <c r="A77" s="2"/>
-      <c r="B77" s="31"/>
-      <c r="C77" s="23"/>
+      <c r="B77" s="17"/>
+      <c r="C77" s="18"/>
       <c r="D77" s="2"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
@@ -2998,8 +3030,8 @@
     </row>
     <row r="78" spans="1:12" ht="16">
       <c r="A78" s="2"/>
-      <c r="B78" s="31"/>
-      <c r="C78" s="23"/>
+      <c r="B78" s="17"/>
+      <c r="C78" s="18"/>
       <c r="D78" s="2"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
@@ -3012,8 +3044,8 @@
     </row>
     <row r="79" spans="1:12" ht="16">
       <c r="A79" s="2"/>
-      <c r="B79" s="31"/>
-      <c r="C79" s="23"/>
+      <c r="B79" s="17"/>
+      <c r="C79" s="18"/>
       <c r="D79" s="2"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
@@ -3026,8 +3058,8 @@
     </row>
     <row r="80" spans="1:12" ht="16">
       <c r="A80" s="2"/>
-      <c r="B80" s="31"/>
-      <c r="C80" s="23"/>
+      <c r="B80" s="17"/>
+      <c r="C80" s="18"/>
       <c r="D80" s="2"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
@@ -3040,8 +3072,8 @@
     </row>
     <row r="81" spans="1:12" ht="16">
       <c r="A81" s="2"/>
-      <c r="B81" s="31"/>
-      <c r="C81" s="23"/>
+      <c r="B81" s="17"/>
+      <c r="C81" s="18"/>
       <c r="D81" s="2"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
@@ -3054,8 +3086,8 @@
     </row>
     <row r="82" spans="1:12" ht="16">
       <c r="A82" s="2"/>
-      <c r="B82" s="31"/>
-      <c r="C82" s="23"/>
+      <c r="B82" s="17"/>
+      <c r="C82" s="18"/>
       <c r="D82" s="2"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
@@ -3068,8 +3100,8 @@
     </row>
     <row r="83" spans="1:12" ht="16">
       <c r="A83" s="2"/>
-      <c r="B83" s="31"/>
-      <c r="C83" s="23"/>
+      <c r="B83" s="17"/>
+      <c r="C83" s="18"/>
       <c r="D83" s="2"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
@@ -3082,8 +3114,8 @@
     </row>
     <row r="84" spans="1:12" ht="16">
       <c r="A84" s="2"/>
-      <c r="B84" s="31"/>
-      <c r="C84" s="23"/>
+      <c r="B84" s="17"/>
+      <c r="C84" s="18"/>
       <c r="D84" s="2"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
@@ -3096,8 +3128,8 @@
     </row>
     <row r="85" spans="1:12" ht="16">
       <c r="A85" s="2"/>
-      <c r="B85" s="31"/>
-      <c r="C85" s="23"/>
+      <c r="B85" s="17"/>
+      <c r="C85" s="18"/>
       <c r="D85" s="2"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
@@ -3110,6 +3142,26 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="D67:G67"/>
+    <mergeCell ref="D68:G68"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="B80:C80"/>
     <mergeCell ref="B74:C74"/>
@@ -3117,26 +3169,6 @@
     <mergeCell ref="B76:C76"/>
     <mergeCell ref="B77:C77"/>
     <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="A66:G66"/>
-    <mergeCell ref="D67:G67"/>
-    <mergeCell ref="D68:G68"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:G2"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="A6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="A7:Z7">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">

</xml_diff>

<commit_message>
cap nhat phan giao
</commit_message>
<xml_diff>
--- a/phan_giao.xlsx
+++ b/phan_giao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pxvanhanh/TPM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30669321-2531-1748-89AC-F74A15333BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF910958-7D51-4443-BC9B-E4A0ED904523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11800" yWindow="600" windowWidth="17000" windowHeight="16180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PHÂN GIAO" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="159">
   <si>
     <t>CÔNG TY THỦY ĐIỆN BẢN VẼ
  PHÂN XƯỞNG VẬN HÀNH</t>
@@ -362,9 +362,6 @@
   </si>
   <si>
     <t>BM.P4.15.36</t>
-  </si>
-  <si>
-    <t>Vi Văn Nhàn</t>
   </si>
   <si>
     <t>HỆ THỐNG NKT H1</t>
@@ -815,34 +812,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -853,6 +822,34 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1105,17 +1102,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="16">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="22" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
       <c r="H1" s="2"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -1123,13 +1120,13 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:26" ht="16">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
       <c r="H2" s="2"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
@@ -1142,12 +1139,12 @@
         <v>2</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
+        <v>156</v>
+      </c>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
       <c r="H3" s="2"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -1173,12 +1170,12 @@
       <c r="B5" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1188,12 +1185,12 @@
       <c r="A6" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
       <c r="H6" s="5"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
@@ -1213,10 +1210,10 @@
       <c r="D7" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="29" t="s">
+      <c r="F7" s="19" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="10" t="s">
@@ -1249,16 +1246,16 @@
       <c r="B8" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="E8" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="30" t="s">
+      <c r="F8" s="20" t="s">
         <v>16</v>
       </c>
       <c r="G8" s="15">
@@ -1277,16 +1274,16 @@
       <c r="B9" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="30" t="s">
+      <c r="F9" s="20" t="s">
         <v>47</v>
       </c>
       <c r="G9" s="16">
@@ -1305,16 +1302,16 @@
       <c r="B10" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="30" t="s">
+      <c r="D10" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="30" t="s">
+      <c r="E10" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="30" t="s">
+      <c r="F10" s="20" t="s">
         <v>47</v>
       </c>
       <c r="G10" s="16">
@@ -1333,16 +1330,16 @@
       <c r="B11" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="30" t="s">
+      <c r="D11" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="F11" s="30" t="s">
+      <c r="E11" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="F11" s="20" t="s">
         <v>26</v>
       </c>
       <c r="G11" s="16">
@@ -1361,16 +1358,16 @@
       <c r="B12" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="F12" s="30" t="s">
+      <c r="E12" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="F12" s="20" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="16">
@@ -1389,16 +1386,16 @@
       <c r="B13" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="30" t="s">
+      <c r="E13" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="F13" s="30" t="s">
+      <c r="F13" s="20" t="s">
         <v>37</v>
       </c>
       <c r="G13" s="16">
@@ -1417,16 +1414,16 @@
       <c r="B14" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="30" t="s">
+      <c r="D14" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="30" t="s">
+      <c r="E14" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="F14" s="30" t="s">
+      <c r="F14" s="20" t="s">
         <v>37</v>
       </c>
       <c r="G14" s="16">
@@ -1445,16 +1442,16 @@
       <c r="B15" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="30" t="s">
+      <c r="D15" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="30" t="s">
+      <c r="E15" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="30" t="s">
+      <c r="F15" s="20" t="s">
         <v>31</v>
       </c>
       <c r="G15" s="16">
@@ -1473,16 +1470,16 @@
       <c r="B16" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="28" t="s">
+      <c r="C16" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="30" t="s">
+      <c r="D16" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="30" t="s">
+      <c r="E16" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="30" t="s">
+      <c r="F16" s="20" t="s">
         <v>31</v>
       </c>
       <c r="G16" s="16">
@@ -1501,16 +1498,16 @@
       <c r="B17" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="30" t="s">
+      <c r="D17" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E17" s="30" t="s">
-        <v>153</v>
-      </c>
-      <c r="F17" s="30" t="s">
+      <c r="E17" s="20" t="s">
+        <v>152</v>
+      </c>
+      <c r="F17" s="20" t="s">
         <v>42</v>
       </c>
       <c r="G17" s="16">
@@ -1529,16 +1526,16 @@
       <c r="B18" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="30" t="s">
+      <c r="D18" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="30" t="s">
-        <v>153</v>
-      </c>
-      <c r="F18" s="30" t="s">
+      <c r="E18" s="20" t="s">
+        <v>152</v>
+      </c>
+      <c r="F18" s="20" t="s">
         <v>42</v>
       </c>
       <c r="G18" s="16">
@@ -1557,16 +1554,16 @@
       <c r="B19" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="30" t="s">
+      <c r="D19" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E19" s="30" t="s">
+      <c r="E19" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="F19" s="30" t="s">
+      <c r="F19" s="20" t="s">
         <v>16</v>
       </c>
       <c r="G19" s="16">
@@ -1585,16 +1582,16 @@
       <c r="B20" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E20" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="F20" s="30" t="s">
+      <c r="D20" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="F20" s="20" t="s">
         <v>15</v>
       </c>
       <c r="G20" s="16">
@@ -1613,16 +1610,16 @@
       <c r="B21" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E21" s="30" t="s">
+      <c r="D21" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E21" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F21" s="30" t="s">
+      <c r="F21" s="20" t="s">
         <v>47</v>
       </c>
       <c r="G21" s="16">
@@ -1641,16 +1638,16 @@
       <c r="B22" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="28" t="s">
+      <c r="C22" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E22" s="30" t="s">
+      <c r="D22" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E22" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F22" s="30" t="s">
+      <c r="F22" s="20" t="s">
         <v>47</v>
       </c>
       <c r="G22" s="16">
@@ -1669,17 +1666,17 @@
       <c r="B23" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D23" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E23" s="30" t="s">
+      <c r="D23" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E23" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="F23" s="30" t="s">
-        <v>152</v>
+      <c r="F23" s="20" t="s">
+        <v>151</v>
       </c>
       <c r="G23" s="16">
         <v>1</v>
@@ -1697,17 +1694,17 @@
       <c r="B24" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="D24" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E24" s="30" t="s">
+      <c r="D24" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E24" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="F24" s="30" t="s">
-        <v>152</v>
+      <c r="F24" s="20" t="s">
+        <v>151</v>
       </c>
       <c r="G24" s="16">
         <v>1</v>
@@ -1725,16 +1722,16 @@
       <c r="B25" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="28" t="s">
+      <c r="C25" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="D25" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E25" s="30" t="s">
+      <c r="D25" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E25" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="F25" s="30" t="s">
+      <c r="F25" s="20" t="s">
         <v>36</v>
       </c>
       <c r="G25" s="16">
@@ -1753,16 +1750,16 @@
       <c r="B26" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E26" s="30" t="s">
+      <c r="D26" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E26" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="F26" s="30" t="s">
+      <c r="F26" s="20" t="s">
         <v>36</v>
       </c>
       <c r="G26" s="16">
@@ -1781,17 +1778,17 @@
       <c r="B27" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="D27" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E27" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="F27" s="30" t="s">
-        <v>154</v>
+      <c r="D27" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E27" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="F27" s="20" t="s">
+        <v>153</v>
       </c>
       <c r="G27" s="16">
         <v>2</v>
@@ -1809,16 +1806,16 @@
       <c r="B28" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="D28" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>154</v>
-      </c>
-      <c r="F28" s="30" t="s">
+      <c r="D28" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" s="20" t="s">
         <v>19</v>
       </c>
       <c r="G28" s="16">
@@ -1837,17 +1834,17 @@
       <c r="B29" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E29" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="F29" s="30" t="s">
-        <v>153</v>
+      <c r="D29" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="F29" s="20" t="s">
+        <v>152</v>
       </c>
       <c r="G29" s="16">
         <v>3</v>
@@ -1865,17 +1862,17 @@
       <c r="B30" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="28" t="s">
+      <c r="C30" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E30" s="30" t="s">
+      <c r="D30" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E30" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="F30" s="30" t="s">
-        <v>153</v>
+      <c r="F30" s="20" t="s">
+        <v>152</v>
       </c>
       <c r="G30" s="16">
         <v>5</v>
@@ -1893,16 +1890,16 @@
       <c r="B31" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="D31" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E31" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="F31" s="30" t="s">
+      <c r="D31" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="F31" s="20" t="s">
         <v>15</v>
       </c>
       <c r="G31" s="16">
@@ -1921,16 +1918,16 @@
       <c r="B32" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D32" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E32" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="F32" s="30" t="s">
+      <c r="D32" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="F32" s="20" t="s">
         <v>15</v>
       </c>
       <c r="G32" s="16">
@@ -1949,16 +1946,16 @@
       <c r="B33" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D33" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E33" s="30" t="s">
+      <c r="D33" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E33" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="F33" s="30" t="s">
+      <c r="F33" s="20" t="s">
         <v>25</v>
       </c>
       <c r="G33" s="16">
@@ -1977,16 +1974,16 @@
       <c r="B34" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="C34" s="28" t="s">
+      <c r="C34" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="D34" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E34" s="30" t="s">
+      <c r="D34" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E34" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="F34" s="30" t="s">
+      <c r="F34" s="20" t="s">
         <v>25</v>
       </c>
       <c r="G34" s="16">
@@ -2005,16 +2002,16 @@
       <c r="B35" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="C35" s="28" t="s">
+      <c r="C35" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="D35" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E35" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="F35" s="30" t="s">
+      <c r="D35" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E35" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="F35" s="20" t="s">
         <v>74</v>
       </c>
       <c r="G35" s="16">
@@ -2033,16 +2030,16 @@
       <c r="B36" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="C36" s="28" t="s">
+      <c r="C36" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D36" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E36" s="30" t="s">
+      <c r="D36" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E36" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F36" s="30" t="s">
+      <c r="F36" s="20" t="s">
         <v>37</v>
       </c>
       <c r="G36" s="16">
@@ -2061,16 +2058,16 @@
       <c r="B37" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C37" s="28" t="s">
+      <c r="C37" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="D37" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E37" s="30" t="s">
+      <c r="D37" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E37" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F37" s="30" t="s">
+      <c r="F37" s="20" t="s">
         <v>50</v>
       </c>
       <c r="G37" s="16">
@@ -2089,17 +2086,17 @@
       <c r="B38" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="C38" s="28" t="s">
+      <c r="C38" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="D38" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E38" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="F38" s="30" t="s">
-        <v>154</v>
+      <c r="D38" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E38" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="F38" s="20" t="s">
+        <v>153</v>
       </c>
       <c r="G38" s="16">
         <v>4</v>
@@ -2117,17 +2114,17 @@
       <c r="B39" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="C39" s="28" t="s">
+      <c r="C39" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="D39" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E39" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="F39" s="30" t="s">
-        <v>154</v>
+      <c r="D39" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E39" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="F39" s="20" t="s">
+        <v>153</v>
       </c>
       <c r="G39" s="16">
         <v>4</v>
@@ -2145,17 +2142,17 @@
       <c r="B40" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="C40" s="28" t="s">
+      <c r="C40" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="D40" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E40" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="F40" s="30" t="s">
-        <v>74</v>
+      <c r="D40" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E40" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="F40" s="20" t="s">
+        <v>151</v>
       </c>
       <c r="G40" s="16">
         <v>1</v>
@@ -2173,17 +2170,17 @@
       <c r="B41" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C41" s="28" t="s">
+      <c r="C41" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="D41" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E41" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="F41" s="30" t="s">
-        <v>153</v>
+      <c r="D41" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E41" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="F41" s="20" t="s">
+        <v>152</v>
       </c>
       <c r="G41" s="16">
         <v>1</v>
@@ -2201,17 +2198,17 @@
       <c r="B42" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="C42" s="28" t="s">
+      <c r="C42" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D42" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E42" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="F42" s="30" t="s">
-        <v>153</v>
+      <c r="D42" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E42" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="F42" s="20" t="s">
+        <v>152</v>
       </c>
       <c r="G42" s="16">
         <v>3</v>
@@ -2229,16 +2226,16 @@
       <c r="B43" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="C43" s="28" t="s">
+      <c r="C43" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D43" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E43" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="F43" s="30" t="s">
+      <c r="D43" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E43" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="F43" s="20" t="s">
         <v>50</v>
       </c>
       <c r="G43" s="16">
@@ -2255,18 +2252,18 @@
         <v>37</v>
       </c>
       <c r="B44" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="C44" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="C44" s="28" t="s">
-        <v>104</v>
-      </c>
-      <c r="D44" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E44" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="F44" s="30" t="s">
+      <c r="D44" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E44" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="F44" s="20" t="s">
         <v>16</v>
       </c>
       <c r="G44" s="16">
@@ -2283,18 +2280,18 @@
         <v>38</v>
       </c>
       <c r="B45" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C45" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="C45" s="28" t="s">
-        <v>107</v>
-      </c>
-      <c r="D45" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E45" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="F45" s="30" t="s">
+      <c r="D45" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E45" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="F45" s="20" t="s">
         <v>16</v>
       </c>
       <c r="G45" s="16">
@@ -2311,18 +2308,18 @@
         <v>39</v>
       </c>
       <c r="B46" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C46" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="C46" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="D46" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E46" s="30" t="s">
+      <c r="D46" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E46" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="F46" s="30" t="s">
+      <c r="F46" s="20" t="s">
         <v>53</v>
       </c>
       <c r="G46" s="16">
@@ -2339,18 +2336,18 @@
         <v>40</v>
       </c>
       <c r="B47" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="C47" s="28" t="s">
-        <v>111</v>
-      </c>
-      <c r="D47" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E47" s="30" t="s">
+      <c r="D47" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E47" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="F47" s="30" t="s">
+      <c r="F47" s="20" t="s">
         <v>53</v>
       </c>
       <c r="G47" s="16">
@@ -2367,18 +2364,18 @@
         <v>41</v>
       </c>
       <c r="B48" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C48" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="C48" s="28" t="s">
+      <c r="D48" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E48" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="D48" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E48" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="F48" s="30" t="s">
+      <c r="F48" s="20" t="s">
         <v>74</v>
       </c>
       <c r="G48" s="16">
@@ -2395,18 +2392,18 @@
         <v>42</v>
       </c>
       <c r="B49" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="C49" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="C49" s="28" t="s">
-        <v>116</v>
-      </c>
-      <c r="D49" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E49" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="F49" s="30" t="s">
+      <c r="D49" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E49" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="F49" s="20" t="s">
         <v>74</v>
       </c>
       <c r="G49" s="16">
@@ -2423,19 +2420,19 @@
         <v>43</v>
       </c>
       <c r="B50" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="C50" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="C50" s="28" t="s">
-        <v>118</v>
-      </c>
-      <c r="D50" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E50" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="F50" s="30" t="s">
-        <v>156</v>
+      <c r="D50" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E50" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="F50" s="20" t="s">
+        <v>155</v>
       </c>
       <c r="G50" s="16">
         <v>1</v>
@@ -2451,19 +2448,19 @@
         <v>44</v>
       </c>
       <c r="B51" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C51" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="C51" s="28" t="s">
-        <v>121</v>
-      </c>
-      <c r="D51" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E51" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="F51" s="30" t="s">
-        <v>156</v>
+      <c r="D51" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E51" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="F51" s="20" t="s">
+        <v>155</v>
       </c>
       <c r="G51" s="16">
         <v>1</v>
@@ -2479,18 +2476,18 @@
         <v>45</v>
       </c>
       <c r="B52" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C52" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="C52" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="D52" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E52" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="F52" s="30" t="s">
+      <c r="D52" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E52" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="F52" s="20" t="s">
         <v>97</v>
       </c>
       <c r="G52" s="16">
@@ -2507,19 +2504,19 @@
         <v>46</v>
       </c>
       <c r="B53" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="C53" s="28" t="s">
-        <v>125</v>
-      </c>
-      <c r="D53" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E53" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="F53" s="30" t="s">
+      <c r="D53" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E53" s="20" t="s">
         <v>97</v>
+      </c>
+      <c r="F53" s="20" t="s">
+        <v>153</v>
       </c>
       <c r="G53" s="16">
         <v>3</v>
@@ -2535,18 +2532,18 @@
         <v>47</v>
       </c>
       <c r="B54" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C54" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="C54" s="28" t="s">
-        <v>128</v>
-      </c>
-      <c r="D54" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E54" s="30" t="s">
+      <c r="D54" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E54" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F54" s="30" t="s">
+      <c r="F54" s="20" t="s">
         <v>50</v>
       </c>
       <c r="G54" s="16">
@@ -2563,18 +2560,18 @@
         <v>48</v>
       </c>
       <c r="B55" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="C55" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="C55" s="28" t="s">
-        <v>130</v>
-      </c>
-      <c r="D55" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E55" s="30" t="s">
-        <v>81</v>
-      </c>
-      <c r="F55" s="30" t="s">
+      <c r="D55" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E55" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="F55" s="20" t="s">
         <v>50</v>
       </c>
       <c r="G55" s="16">
@@ -2591,18 +2588,18 @@
         <v>49</v>
       </c>
       <c r="B56" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C56" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="C56" s="28" t="s">
-        <v>132</v>
-      </c>
-      <c r="D56" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E56" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="F56" s="30" t="s">
+      <c r="D56" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E56" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="F56" s="20" t="s">
         <v>15</v>
       </c>
       <c r="G56" s="16">
@@ -2619,19 +2616,19 @@
         <v>50</v>
       </c>
       <c r="B57" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="C57" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="C57" s="28" t="s">
-        <v>134</v>
-      </c>
-      <c r="D57" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E57" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="F57" s="30" t="s">
+      <c r="D57" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E57" s="20" t="s">
         <v>97</v>
+      </c>
+      <c r="F57" s="20" t="s">
+        <v>74</v>
       </c>
       <c r="G57" s="16">
         <v>1</v>
@@ -2647,18 +2644,18 @@
         <v>51</v>
       </c>
       <c r="B58" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C58" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="C58" s="28" t="s">
-        <v>136</v>
-      </c>
-      <c r="D58" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E58" s="30" t="s">
+      <c r="D58" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E58" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="F58" s="30" t="s">
+      <c r="F58" s="20" t="s">
         <v>53</v>
       </c>
       <c r="G58" s="16">
@@ -2675,18 +2672,18 @@
         <v>52</v>
       </c>
       <c r="B59" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C59" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="C59" s="28" t="s">
-        <v>138</v>
-      </c>
-      <c r="D59" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E59" s="30" t="s">
+      <c r="D59" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E59" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F59" s="30" t="s">
+      <c r="F59" s="20" t="s">
         <v>31</v>
       </c>
       <c r="G59" s="16">
@@ -2703,18 +2700,18 @@
         <v>53</v>
       </c>
       <c r="B60" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="C60" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="C60" s="28" t="s">
-        <v>140</v>
-      </c>
-      <c r="D60" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E60" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="F60" s="30" t="s">
+      <c r="D60" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E60" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="F60" s="20" t="s">
         <v>74</v>
       </c>
       <c r="G60" s="16">
@@ -2731,19 +2728,19 @@
         <v>54</v>
       </c>
       <c r="B61" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="C61" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="C61" s="28" t="s">
-        <v>142</v>
-      </c>
-      <c r="D61" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E61" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="F61" s="30" t="s">
-        <v>153</v>
+      <c r="D61" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E61" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="F61" s="20" t="s">
+        <v>152</v>
       </c>
       <c r="G61" s="16">
         <v>4</v>
@@ -2759,19 +2756,19 @@
         <v>55</v>
       </c>
       <c r="B62" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="C62" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="C62" s="28" t="s">
-        <v>144</v>
-      </c>
-      <c r="D62" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E62" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="F62" s="30" t="s">
-        <v>153</v>
+      <c r="D62" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E62" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="F62" s="20" t="s">
+        <v>152</v>
       </c>
       <c r="G62" s="16">
         <v>1</v>
@@ -2787,18 +2784,18 @@
         <v>56</v>
       </c>
       <c r="B63" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C63" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C63" s="28" t="s">
-        <v>146</v>
-      </c>
-      <c r="D63" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E63" s="30" t="s">
-        <v>154</v>
-      </c>
-      <c r="F63" s="30" t="s">
+      <c r="D63" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E63" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="F63" s="20" t="s">
         <v>19</v>
       </c>
       <c r="G63" s="16">
@@ -2815,18 +2812,18 @@
         <v>57</v>
       </c>
       <c r="B64" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C64" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="C64" s="28" t="s">
-        <v>148</v>
-      </c>
-      <c r="D64" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E64" s="30" t="s">
-        <v>154</v>
-      </c>
-      <c r="F64" s="30" t="s">
+      <c r="D64" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E64" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="F64" s="20" t="s">
         <v>19</v>
       </c>
       <c r="G64" s="16">
@@ -2853,15 +2850,15 @@
       <c r="L65" s="3"/>
     </row>
     <row r="66" spans="1:12" ht="186.75" customHeight="1">
-      <c r="A66" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="B66" s="18"/>
-      <c r="C66" s="18"/>
-      <c r="D66" s="18"/>
-      <c r="E66" s="18"/>
-      <c r="F66" s="18"/>
-      <c r="G66" s="18"/>
+      <c r="A66" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B66" s="22"/>
+      <c r="C66" s="22"/>
+      <c r="D66" s="22"/>
+      <c r="E66" s="22"/>
+      <c r="F66" s="22"/>
+      <c r="G66" s="22"/>
       <c r="H66" s="2"/>
       <c r="I66" s="3"/>
       <c r="J66" s="3"/>
@@ -2869,17 +2866,17 @@
       <c r="L66" s="3"/>
     </row>
     <row r="67" spans="1:12" ht="16">
-      <c r="A67" s="21" t="s">
-        <v>150</v>
-      </c>
-      <c r="B67" s="18"/>
-      <c r="C67" s="18"/>
-      <c r="D67" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="E67" s="18"/>
-      <c r="F67" s="18"/>
-      <c r="G67" s="18"/>
+      <c r="A67" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="B67" s="22"/>
+      <c r="C67" s="22"/>
+      <c r="D67" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="E67" s="22"/>
+      <c r="F67" s="22"/>
+      <c r="G67" s="22"/>
       <c r="H67" s="2"/>
       <c r="I67" s="3"/>
       <c r="J67" s="3"/>
@@ -2887,15 +2884,15 @@
       <c r="L67" s="4"/>
     </row>
     <row r="68" spans="1:12" ht="16">
-      <c r="A68" s="17"/>
-      <c r="B68" s="18"/>
-      <c r="C68" s="18"/>
-      <c r="D68" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="E68" s="18"/>
-      <c r="F68" s="18"/>
-      <c r="G68" s="18"/>
+      <c r="A68" s="30"/>
+      <c r="B68" s="22"/>
+      <c r="C68" s="22"/>
+      <c r="D68" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="E68" s="22"/>
+      <c r="F68" s="22"/>
+      <c r="G68" s="22"/>
       <c r="H68" s="2"/>
       <c r="I68" s="3"/>
       <c r="J68" s="3"/>
@@ -2904,8 +2901,8 @@
     </row>
     <row r="69" spans="1:12" ht="16">
       <c r="A69" s="2"/>
-      <c r="B69" s="17"/>
-      <c r="C69" s="18"/>
+      <c r="B69" s="30"/>
+      <c r="C69" s="22"/>
       <c r="D69" s="2"/>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
@@ -2918,8 +2915,8 @@
     </row>
     <row r="70" spans="1:12" ht="16">
       <c r="A70" s="2"/>
-      <c r="B70" s="17"/>
-      <c r="C70" s="18"/>
+      <c r="B70" s="30"/>
+      <c r="C70" s="22"/>
       <c r="D70" s="2"/>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
@@ -2932,8 +2929,8 @@
     </row>
     <row r="71" spans="1:12" ht="16">
       <c r="A71" s="2"/>
-      <c r="B71" s="17"/>
-      <c r="C71" s="18"/>
+      <c r="B71" s="30"/>
+      <c r="C71" s="22"/>
       <c r="D71" s="2"/>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
@@ -2946,8 +2943,8 @@
     </row>
     <row r="72" spans="1:12" ht="16">
       <c r="A72" s="2"/>
-      <c r="B72" s="17"/>
-      <c r="C72" s="18"/>
+      <c r="B72" s="30"/>
+      <c r="C72" s="22"/>
       <c r="D72" s="2"/>
       <c r="E72" s="3"/>
       <c r="F72" s="4"/>
@@ -2960,8 +2957,8 @@
     </row>
     <row r="73" spans="1:12" ht="16">
       <c r="A73" s="2"/>
-      <c r="B73" s="17"/>
-      <c r="C73" s="18"/>
+      <c r="B73" s="30"/>
+      <c r="C73" s="22"/>
       <c r="D73" s="2"/>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
@@ -2974,8 +2971,8 @@
     </row>
     <row r="74" spans="1:12" ht="16">
       <c r="A74" s="2"/>
-      <c r="B74" s="17"/>
-      <c r="C74" s="18"/>
+      <c r="B74" s="30"/>
+      <c r="C74" s="22"/>
       <c r="D74" s="2"/>
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
@@ -2988,8 +2985,8 @@
     </row>
     <row r="75" spans="1:12" ht="16">
       <c r="A75" s="2"/>
-      <c r="B75" s="17"/>
-      <c r="C75" s="18"/>
+      <c r="B75" s="30"/>
+      <c r="C75" s="22"/>
       <c r="D75" s="2"/>
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
@@ -3002,8 +2999,8 @@
     </row>
     <row r="76" spans="1:12" ht="16">
       <c r="A76" s="2"/>
-      <c r="B76" s="17"/>
-      <c r="C76" s="18"/>
+      <c r="B76" s="30"/>
+      <c r="C76" s="22"/>
       <c r="D76" s="2"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
@@ -3016,8 +3013,8 @@
     </row>
     <row r="77" spans="1:12" ht="16">
       <c r="A77" s="2"/>
-      <c r="B77" s="17"/>
-      <c r="C77" s="18"/>
+      <c r="B77" s="30"/>
+      <c r="C77" s="22"/>
       <c r="D77" s="2"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
@@ -3030,8 +3027,8 @@
     </row>
     <row r="78" spans="1:12" ht="16">
       <c r="A78" s="2"/>
-      <c r="B78" s="17"/>
-      <c r="C78" s="18"/>
+      <c r="B78" s="30"/>
+      <c r="C78" s="22"/>
       <c r="D78" s="2"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
@@ -3044,8 +3041,8 @@
     </row>
     <row r="79" spans="1:12" ht="16">
       <c r="A79" s="2"/>
-      <c r="B79" s="17"/>
-      <c r="C79" s="18"/>
+      <c r="B79" s="30"/>
+      <c r="C79" s="22"/>
       <c r="D79" s="2"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
@@ -3058,8 +3055,8 @@
     </row>
     <row r="80" spans="1:12" ht="16">
       <c r="A80" s="2"/>
-      <c r="B80" s="17"/>
-      <c r="C80" s="18"/>
+      <c r="B80" s="30"/>
+      <c r="C80" s="22"/>
       <c r="D80" s="2"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
@@ -3072,8 +3069,8 @@
     </row>
     <row r="81" spans="1:12" ht="16">
       <c r="A81" s="2"/>
-      <c r="B81" s="17"/>
-      <c r="C81" s="18"/>
+      <c r="B81" s="30"/>
+      <c r="C81" s="22"/>
       <c r="D81" s="2"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
@@ -3086,8 +3083,8 @@
     </row>
     <row r="82" spans="1:12" ht="16">
       <c r="A82" s="2"/>
-      <c r="B82" s="17"/>
-      <c r="C82" s="18"/>
+      <c r="B82" s="30"/>
+      <c r="C82" s="22"/>
       <c r="D82" s="2"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
@@ -3100,8 +3097,8 @@
     </row>
     <row r="83" spans="1:12" ht="16">
       <c r="A83" s="2"/>
-      <c r="B83" s="17"/>
-      <c r="C83" s="18"/>
+      <c r="B83" s="30"/>
+      <c r="C83" s="22"/>
       <c r="D83" s="2"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
@@ -3114,8 +3111,8 @@
     </row>
     <row r="84" spans="1:12" ht="16">
       <c r="A84" s="2"/>
-      <c r="B84" s="17"/>
-      <c r="C84" s="18"/>
+      <c r="B84" s="30"/>
+      <c r="C84" s="22"/>
       <c r="D84" s="2"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
@@ -3128,8 +3125,8 @@
     </row>
     <row r="85" spans="1:12" ht="16">
       <c r="A85" s="2"/>
-      <c r="B85" s="17"/>
-      <c r="C85" s="18"/>
+      <c r="B85" s="30"/>
+      <c r="C85" s="22"/>
       <c r="D85" s="2"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
@@ -3142,26 +3139,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:G2"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A66:G66"/>
-    <mergeCell ref="D67:G67"/>
-    <mergeCell ref="D68:G68"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="B80:C80"/>
     <mergeCell ref="B74:C74"/>
@@ -3169,6 +3146,26 @@
     <mergeCell ref="B76:C76"/>
     <mergeCell ref="B77:C77"/>
     <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="D67:G67"/>
+    <mergeCell ref="D68:G68"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="A6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="A7:Z7">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">

</xml_diff>